<commit_message>
add logs and new README
</commit_message>
<xml_diff>
--- a/Результат/reconciliation.xlsx
+++ b/Результат/reconciliation.xlsx
@@ -5074,9 +5074,8 @@
           <t>Итого записей:</t>
         </is>
       </c>
-      <c r="B119" s="7">
-        <f>COUNTA(A2:A117)</f>
-        <v/>
+      <c r="B119" s="7" t="n">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -5507,9 +5506,8 @@
           <t>Итого записей:</t>
         </is>
       </c>
-      <c r="B13" s="7">
-        <f>COUNTA(A2:A11)</f>
-        <v/>
+      <c r="B13" s="7" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -5735,9 +5733,8 @@
           <t>Итого записей:</t>
         </is>
       </c>
-      <c r="B8" s="7">
-        <f>COUNTA(A2:A6)</f>
-        <v/>
+      <c r="B8" s="7" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>